<commit_message>
Populate database and correct direct plan classifications
</commit_message>
<xml_diff>
--- a/TransactionsLatestCAS.xlsx
+++ b/TransactionsLatestCAS.xlsx
@@ -8351,16 +8351,16 @@
         <v>41997.9</v>
       </c>
       <c r="I2" t="n">
-        <v>22.6309</v>
+        <v>22.5431</v>
       </c>
       <c r="J2" t="n">
-        <v>48593.91</v>
+        <v>48405.38</v>
       </c>
       <c r="K2" t="n">
-        <v>15.71</v>
+        <v>15.26</v>
       </c>
       <c r="L2" t="n">
-        <v>9.98</v>
+        <v>9.68</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
@@ -8406,16 +8406,16 @@
         <v>41997.9</v>
       </c>
       <c r="I3" t="n">
-        <v>12.5355</v>
+        <v>12.5017</v>
       </c>
       <c r="J3" t="n">
-        <v>54600.01</v>
+        <v>54452.79</v>
       </c>
       <c r="K3" t="n">
-        <v>30.01</v>
+        <v>29.66</v>
       </c>
       <c r="L3" t="n">
-        <v>18.32</v>
+        <v>18.08</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
@@ -8461,16 +8461,16 @@
         <v>39998</v>
       </c>
       <c r="I4" t="n">
-        <v>154.523</v>
+        <v>155.074</v>
       </c>
       <c r="J4" t="n">
-        <v>45995.32</v>
+        <v>46159.33</v>
       </c>
       <c r="K4" t="n">
-        <v>14.99</v>
+        <v>15.4</v>
       </c>
       <c r="L4" t="n">
-        <v>5.97</v>
+        <v>6.12</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
@@ -8516,16 +8516,16 @@
         <v>41997.9</v>
       </c>
       <c r="I5" t="n">
-        <v>4975.989</v>
+        <v>4955.5286</v>
       </c>
       <c r="J5" t="n">
-        <v>49595.68</v>
+        <v>49391.75</v>
       </c>
       <c r="K5" t="n">
-        <v>18.09</v>
+        <v>17.61</v>
       </c>
       <c r="L5" t="n">
-        <v>11.58</v>
+        <v>11.26</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
@@ -8571,16 +8571,16 @@
         <v>41997.9</v>
       </c>
       <c r="I6" t="n">
-        <v>46.7087</v>
+        <v>46.5163</v>
       </c>
       <c r="J6" t="n">
-        <v>47662.49</v>
+        <v>47466.16</v>
       </c>
       <c r="K6" t="n">
-        <v>13.49</v>
+        <v>13.02</v>
       </c>
       <c r="L6" t="n">
-        <v>8.529999999999999</v>
+        <v>8.23</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
@@ -8626,16 +8626,16 @@
         <v>41997.9</v>
       </c>
       <c r="I7" t="n">
-        <v>16.7853</v>
+        <v>16.9349</v>
       </c>
       <c r="J7" t="n">
-        <v>47044.4</v>
+        <v>47463.68</v>
       </c>
       <c r="K7" t="n">
-        <v>12.02</v>
+        <v>13.01</v>
       </c>
       <c r="L7" t="n">
-        <v>7.78</v>
+        <v>8.390000000000001</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
@@ -8681,16 +8681,16 @@
         <v>41997.9</v>
       </c>
       <c r="I8" t="n">
-        <v>168.616</v>
+        <v>169.225</v>
       </c>
       <c r="J8" t="n">
-        <v>43529.57</v>
+        <v>43686.79</v>
       </c>
       <c r="K8" t="n">
-        <v>3.65</v>
+        <v>4.02</v>
       </c>
       <c r="L8" t="n">
-        <v>2.36</v>
+        <v>2.59</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
@@ -8736,16 +8736,16 @@
         <v>41997.9</v>
       </c>
       <c r="I9" t="n">
-        <v>11.747</v>
+        <v>11.748</v>
       </c>
       <c r="J9" t="n">
-        <v>47847.67</v>
+        <v>47851.74</v>
       </c>
       <c r="K9" t="n">
-        <v>13.93</v>
+        <v>13.94</v>
       </c>
       <c r="L9" t="n">
-        <v>8.76</v>
+        <v>8.75</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
@@ -8791,16 +8791,16 @@
         <v>41997.9</v>
       </c>
       <c r="I10" t="n">
-        <v>27.8205</v>
+        <v>27.732</v>
       </c>
       <c r="J10" t="n">
-        <v>48767.42</v>
+        <v>48612.28</v>
       </c>
       <c r="K10" t="n">
-        <v>16.12</v>
+        <v>15.75</v>
       </c>
       <c r="L10" t="n">
-        <v>9.99</v>
+        <v>9.75</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>

</xml_diff>